<commit_message>
Corrige BIO 2 : cellules de correction decalees + retire les colonnes Erreur/Correction du fichier telecharge
Une stagiaire a signale que la cellule S8 etait notee comme si c etait
un montant HT alors que c est un PU dans le tableau. Le fichier de
correction utilise en realite une mise en page decalee d une colonne
par rapport au fichier vierge sur le bloc de droite (mais pas sur le
bloc de gauche), ce que le generateur de cle ne detectait pas
correctement. La cle de correction est entierement regeneree avec une
methode qui traite les deux blocs separement (26 cellules cibles au
lieu de 91, qui correspondent maintenant exactement aux erreurs
volontairement inserees dans la facture).

Retire aussi les libelles Erreur et Correction du fichier Excel
que les stagiaires telechargent : ils restent uniquement dans le
fichier de correction que la formatrice diffuse ensuite.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/administration-des-ventes/assets/exercices-excel/bio-2.xlsx
+++ b/administration-des-ventes/assets/exercices-excel/bio-2.xlsx
@@ -1,39 +1,489 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nellydoucet\Documents\02. SECRETAIRE COMPTABLE\02. ADMINISTRATION DES VENTES\2023\01. ADMINISTRATION DES VENTES\SC2024\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9D383AA-420D-416B-A2D6-0E437774B251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{31AA7DA7-77DF-4F79-B56E-8A56121FEEEC}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>Feuilles de calcul</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>1</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="1" baseType="lpstr">
+      <vt:lpstr>Feuil1</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <Company/>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>Nelly DOUCET</dc:creator>
+  <cp:lastModifiedBy>Nelly DOUCET</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2024-03-25T15:19:57Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2024-03-25T15:20:43Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\calcChain.xml><?xml version="1.0" encoding="utf-8"?>
+<calcChain xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <c r="D42" i="1" l="1"/>
+  <c r="U37" i="1"/>
+  <c r="V37" i="1" s="1"/>
+  <c r="H37" i="1"/>
+  <c r="I37" i="1" s="1"/>
+  <c r="U36" i="1"/>
+  <c r="V36" i="1" s="1"/>
+  <c r="H36" i="1"/>
+  <c r="I36" i="1" s="1"/>
+  <c r="U35" i="1"/>
+  <c r="V35" i="1" s="1"/>
+  <c r="I35" i="1"/>
+  <c r="V34" i="1"/>
+  <c r="U34" i="1"/>
+  <c r="H34" i="1"/>
+  <c r="I34" i="1" s="1"/>
+  <c r="I38" i="1" s="1"/>
+  <c r="V33" i="1"/>
+  <c r="U33" i="1"/>
+  <c r="I33" i="1"/>
+  <c r="O16" i="1"/>
+  <c r="Q16" i="1" s="1"/>
+  <c r="B16" i="1"/>
+  <c r="D16" i="1" s="1"/>
+  <c r="V11" i="1"/>
+  <c r="I11" i="1"/>
+  <c r="H11" i="1"/>
+  <c r="V10" i="1"/>
+  <c r="O15" i="1" s="1"/>
+  <c r="Q15" i="1" s="1"/>
+  <c r="I10" i="1"/>
+  <c r="H10" i="1"/>
+  <c r="V9" i="1"/>
+  <c r="V12" i="1" s="1"/>
+  <c r="I9" i="1"/>
+  <c r="B15" i="1" s="1"/>
+  <c r="D15" i="1" s="1"/>
+  <c r="I17" i="1" s="1"/>
+  <c r="H9" i="1"/>
+  <c r="V8" i="1"/>
+  <c r="I8" i="1"/>
+  <c r="H8" i="1"/>
+  <c r="V17" i="1" l="1"/>
+  <c r="V18" i="1" s="1"/>
+  <c r="O42" i="1"/>
+  <c r="Q42" i="1" s="1"/>
+  <c r="V43" i="1" s="1"/>
+  <c r="J39" i="1"/>
+  <c r="I40" i="1"/>
+  <c r="B43" i="1"/>
+  <c r="D43" i="1" s="1"/>
+  <c r="I43" i="1" s="1"/>
+  <c r="I12" i="1"/>
+  <c r="V38" i="1"/>
+  <c r="I39" i="1"/>
+  <c r="I41" i="1" l="1"/>
+  <c r="I42" i="1"/>
+  <c r="I44" i="1" s="1"/>
+  <c r="V39" i="1"/>
+  <c r="V40" i="1"/>
+  <c r="K13" i="1"/>
+  <c r="I14" i="1" s="1"/>
+  <c r="K15" i="1" l="1"/>
+  <c r="I16" i="1" s="1"/>
+  <c r="I18" i="1" s="1"/>
+  <c r="V41" i="1"/>
+  <c r="V42" i="1" s="1"/>
+  <c r="V44" i="1" s="1"/>
+</calcChain>
+</file>
+
+<file path=xl\drawings\drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>733425</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>457199</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>361332</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DDB83C7B-35E6-4C82-AFAE-46EB8681DC63}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="18926175" y="8220075"/>
+          <a:ext cx="447674" cy="532782"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>733425</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>7619</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="444341" cy="562928"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C8E7D6B-B583-4B84-8914-A46038BF547A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="18926175" y="13352144"/>
+          <a:ext cx="444341" cy="562928"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>58213</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>142077</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1001233" cy="637954"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="ZoneTexte 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4B1C199-3896-42B6-A850-BD5D7CF5A0CC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="58213" y="3742527"/>
+          <a:ext cx="1001233" cy="637954"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="1100"/>
+            <a:t>(1)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="fr-FR" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="1100"/>
+            <a:t>(2)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>425302</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>159488</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1001233" cy="637954"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="ZoneTexte 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EBE42E9A-71A1-41B4-B1EE-90ED1CA4EE63}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7864327" y="3759938"/>
+          <a:ext cx="1001233" cy="637954"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="1100"/>
+            <a:t>(1)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="fr-FR" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="1100"/>
+            <a:t>(2)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>44303</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>186069</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1001233" cy="637954"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="ZoneTexte 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8A25816-9DE7-41A4-A1FF-F2D61BA9BCD2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="44303" y="12539994"/>
+          <a:ext cx="1001233" cy="637954"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="1100"/>
+            <a:t>(1)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="fr-FR" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="1100"/>
+            <a:t>(2)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>442093</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>165824</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1001233" cy="637954"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="ZoneTexte 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E737FDCE-BFFB-4B16-B834-722B2CDE6BBB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7881118" y="12519749"/>
+          <a:ext cx="1001233" cy="637954"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="1100"/>
+            <a:t>(1)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="fr-FR" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="fr-FR" sz="1100"/>
+            <a:t>(2)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="49">
   <si>
     <t xml:space="preserve">CLIENT : BIOARTIGUES  </t>
@@ -214,7 +664,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="8">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
@@ -1294,381 +1744,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>31</xdr:col>
-      <xdr:colOff>457199</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>361332</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DDB83C7B-35E6-4C82-AFAE-46EB8681DC63}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="18926175" y="8220075"/>
-          <a:ext cx="447674" cy="532782"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>7619</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="444341" cy="562928"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C8E7D6B-B583-4B84-8914-A46038BF547A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="18926175" y="13352144"/>
-          <a:ext cx="444341" cy="562928"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>58213</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>142077</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1001233" cy="637954"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="ZoneTexte 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4B1C199-3896-42B6-A850-BD5D7CF5A0CC}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="58213" y="3742527"/>
-          <a:ext cx="1001233" cy="637954"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="fr-FR" sz="1100"/>
-            <a:t>(1)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="fr-FR" sz="1100"/>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="fr-FR" sz="1100"/>
-            <a:t>(2)</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>425302</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>159488</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1001233" cy="637954"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="ZoneTexte 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EBE42E9A-71A1-41B4-B1EE-90ED1CA4EE63}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7864327" y="3759938"/>
-          <a:ext cx="1001233" cy="637954"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="fr-FR" sz="1100"/>
-            <a:t>(1)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="fr-FR" sz="1100"/>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="fr-FR" sz="1100"/>
-            <a:t>(2)</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>44303</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>186069</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1001233" cy="637954"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="6" name="ZoneTexte 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8A25816-9DE7-41A4-A1FF-F2D61BA9BCD2}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="44303" y="12539994"/>
-          <a:ext cx="1001233" cy="637954"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="fr-FR" sz="1100"/>
-            <a:t>(1)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="fr-FR" sz="1100"/>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="fr-FR" sz="1100"/>
-            <a:t>(2)</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>442093</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>165824</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1001233" cy="637954"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="ZoneTexte 6">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E737FDCE-BFFB-4B16-B834-722B2CDE6BBB}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7881118" y="12519749"/>
-          <a:ext cx="1001233" cy="637954"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="fr-FR" sz="1100"/>
-            <a:t>(1)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="fr-FR" sz="1100"/>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="fr-FR" sz="1100"/>
-            <a:t>(2)</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -1963,7 +2039,41 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nellydoucet\Documents\02. SECRETAIRE COMPTABLE\02. ADMINISTRATION DES VENTES\2023\01. ADMINISTRATION DES VENTES\SC2024\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9D383AA-420D-416B-A2D6-0E437774B251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{31AA7DA7-77DF-4F79-B56E-8A56121FEEEC}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A6B454F-0B21-4808-BC5F-400E7D895E8E}">
   <dimension ref="B2:AMQ1048534"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.85546875" defaultRowHeight="14.1" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3629,32 +3739,20 @@
       <c r="W19" s="62"/>
     </row>
     <row r="20" spans="2:1031" s="8" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="113" t="s">
-        <v>31</v>
-      </c>
       <c r="C20" s="114"/>
       <c r="D20" s="114"/>
       <c r="E20" s="114"/>
       <c r="F20" s="115"/>
-      <c r="G20" s="116" t="s">
-        <v>32</v>
-      </c>
       <c r="H20" s="116"/>
       <c r="I20" s="116"/>
       <c r="J20" s="116"/>
       <c r="K20" s="116"/>
       <c r="L20" s="116"/>
       <c r="M20" s="116"/>
-      <c r="O20" s="113" t="s">
-        <v>31</v>
-      </c>
       <c r="P20" s="114"/>
       <c r="Q20" s="114"/>
       <c r="R20" s="114"/>
       <c r="S20" s="115"/>
-      <c r="T20" s="116" t="s">
-        <v>32</v>
-      </c>
       <c r="U20" s="116"/>
       <c r="V20" s="116"/>
       <c r="W20" s="116"/>
@@ -5449,32 +5547,20 @@
       <c r="W45" s="172"/>
     </row>
     <row r="46" spans="2:26" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="113" t="s">
-        <v>31</v>
-      </c>
       <c r="C46" s="114"/>
       <c r="D46" s="114"/>
       <c r="E46" s="114"/>
       <c r="F46" s="115"/>
-      <c r="G46" s="116" t="s">
-        <v>32</v>
-      </c>
       <c r="H46" s="116"/>
       <c r="I46" s="116"/>
       <c r="J46" s="116"/>
       <c r="K46" s="116"/>
       <c r="L46" s="116"/>
       <c r="M46" s="116"/>
-      <c r="O46" s="113" t="s">
-        <v>31</v>
-      </c>
       <c r="P46" s="114"/>
       <c r="Q46" s="114"/>
       <c r="R46" s="114"/>
       <c r="S46" s="115"/>
-      <c r="T46" s="116" t="s">
-        <v>32</v>
-      </c>
       <c r="U46" s="116"/>
       <c r="V46" s="116"/>
       <c r="W46" s="116"/>

</xml_diff>